<commit_message>
Add dept-specific level channels via Roles sheet
Replaces the Levels sheet with a 3-column Roles sheet
(Department | Level | Channel) so channel assignments are scoped
to a department+level combo. A QC Lead only gets QC Lead channels,
not Recruiting Lead channels. Expected channels for a person =
their department base channels + their dept-level specific channels.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/references/slack-template.xlsx
+++ b/references/slack-template.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="People" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Departments" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Levels" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Roles" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -628,12 +628,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>all-qc</t>
+          <t>announcements</t>
         </is>
       </c>
     </row>
@@ -645,95 +645,119 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>qc-managers</t>
+          <t>all-qc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Recruiting</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>-all-recruiting</t>
+          <t>all-aptel</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>-all-recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Recruiting</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>EStream</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>all-estream</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EStream</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>all-aptel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>EStream</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>--- Available Channels ---</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>-all-recruiting</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr"/>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>-leadership</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>22358-elevate</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>all-aptel</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>all-estream</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>all-managers</t>
-        </is>
-      </c>
+      <c r="B18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr"/>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>all-qc</t>
+          <t>-all-recruiting</t>
         </is>
       </c>
     </row>
@@ -741,7 +765,7 @@
       <c r="A20" s="3" t="inlineStr"/>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>all-swat</t>
+          <t>-leadership</t>
         </is>
       </c>
     </row>
@@ -749,7 +773,7 @@
       <c r="A21" s="3" t="inlineStr"/>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>22358-elevate</t>
         </is>
       </c>
     </row>
@@ -757,7 +781,7 @@
       <c r="A22" s="3" t="inlineStr"/>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>critical-items</t>
+          <t>all-aptel</t>
         </is>
       </c>
     </row>
@@ -765,13 +789,61 @@
       <c r="A23" s="3" t="inlineStr"/>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>development</t>
+          <t>all-estream</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr"/>
       <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>all-managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>all-qc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>all-swat</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>critical-items</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>development</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>qc-managers</t>
         </is>
@@ -788,20 +860,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
@@ -810,10 +888,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>SWAT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>all-swat</t>
         </is>
@@ -822,10 +905,15 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>SWAT</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>all-managers</t>
         </is>
@@ -834,210 +922,183 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>all-aptel</t>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>all-managers</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>qc-managers</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>all-managers</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>qc-managers</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Recruiting</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>--- Available Channels ---</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>-all-recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>-leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>22358-elevate</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
           <t>all-aptel</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>announcements</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Lead</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>all-aptel</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Lead</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>announcements</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>all-aptel</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>announcements</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>--- Available Channels ---</t>
-        </is>
-      </c>
+      <c r="A14" s="3" t="inlineStr"/>
       <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>all-estream</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>-all-recruiting</t>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>all-managers</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>-leadership</t>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>all-qc</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>22358-elevate</t>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>all-swat</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>all-aptel</t>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>all-estream</t>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>critical-items</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr"/>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>all-managers</t>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>development</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>all-qc</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>all-swat</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>announcements</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr"/>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>critical-items</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr"/>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>development</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr"/>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>qc-managers</t>
         </is>

</xml_diff>